<commit_message>
feat(F-NAR-019): TREE-DIF-051 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-051.xlsx
+++ b/stories/arbres/TREE-DIF-051.xlsx
@@ -3275,17 +3275,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Un brin de laine bleue reste au chaud. Le noir entre, puis s'en va. De la neige, sur le métal. Un flocon reste au fer, et le cacao sent le sucre.</t>
+          <t>Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Un fil bleu dort contre le métal. Le noir entre, puis s'en va. De la neige, sur le métal. Un flocon reste au fer, et le cacao sent le sucre.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Un brin de laine bleue reste au chaud. Le noir entre, puis s'en va. De la &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, et le cacao sent le sucre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Un fil bleu dort contre le métal. Le noir entre, puis s'en va. De la &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, et le cacao sent le sucre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Un brin de laine bleue reste au chaud. Le noir entre, puis s'en va. De la &lt;emphasis&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, et le cacao sent le sucre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Un fil bleu dort contre le métal. Le noir entre, puis s'en va. De la &lt;emphasis&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, et le cacao sent le sucre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3427,7 +3427,7 @@
 enfant-f|Vous voyez le trou, tous les deux ?
 papa|Deux places, une seule cabine.
 maman|Le filet les a gardés.
-narrateur|Un brin de laine bleue reste au chaud.
+narrateur|Un fil bleu dort contre le métal.
 narrateur|Le noir entre, puis s'en va.
 enfant-f|De la neige, sur le métal.
 narrateur|Un flocon reste au fer, et le cacao sent le sucre.</t>
@@ -3646,17 +3646,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Un brin de laine bleue reste au chaud. Le noir frappe le verre, un instant. On l'a vu, ensemble. La neige éclaire le manteau, et le sac vide.</t>
+          <t>Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Le châle garde une chaleur de maison. Le noir frappe le verre, un instant. On l'a vu, ensemble. La neige éclaire le manteau, et le sac vide.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Un brin de laine bleue reste au chaud. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le sac vide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Le châle garde une chaleur de maison. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le sac vide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Un brin de laine bleue reste au chaud. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le sac vide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Le châle garde une chaleur de maison. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le sac vide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3798,7 +3798,7 @@
 enfant-f|Vous êtes plus près, maintenant.
 papa|Tu les as repris tous les deux.
 maman|Le filet peut attendre, vide.
-narrateur|Un brin de laine bleue reste au chaud.
+narrateur|Le châle garde une chaleur de maison.
 narrateur|Le noir frappe le verre, un instant.
 enfant-f|On l'a vu, ensemble.
 narrateur|La neige éclaire le manteau, et le sac vide.</t>
@@ -3833,17 +3833,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Le châle glisse sur le vinyle chaud. C'est trop lisse, ici. Le hérisson part vers l'allée, rond. Le renard se faufile sous le siège. Le châle ne les tient plus. Elle attrape l'un, et l'autre disparaît. Ils ne jouent plus au même endroit. On les reprend, les deux. Je ne veux pas choisir. Tu les poses comment, sur le siège ?</t>
+          <t>Le châle glisse sur le vinyle chaud. C'est trop lisse, ici. Le hérisson part vers l'allée, rond. Le renard se faufile sous le siège. Le châle ne les tient plus. Elle attrape l'un, et l'autre disparaît. Ils ne jouent plus au même endroit. Attrape-les ensemble, pas l'un après l'autre. Je ne veux pas choisir. Tu les poses comment, sur le siège ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le châle glisse sur le vinyle chaud. C'est trop lisse, ici. Le hérisson part vers l'allée, rond. Le renard se faufile sous le siège. Le châle ne les tient plus. Elle attrape l'un, et l'autre disparaît. Ils ne jouent plus au même endroit. On les reprend, les deux. Je ne veux pas choisir. Tu les poses comment, sur le siège ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le châle glisse sur le vinyle chaud. C'est trop lisse, ici. Le hérisson part vers l'allée, rond. Le renard se faufile sous le siège. Le châle ne les tient plus. Elle attrape l'un, et l'autre disparaît. Ils ne jouent plus au même endroit. Attrape-les ensemble, pas l'un après l'autre. Je ne veux pas choisir. Tu les poses comment, sur le siège ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le châle glisse sur le vinyle chaud. C'est trop lisse, ici. Le hérisson part vers l'allée, rond. Le renard se faufile sous le siège. Le châle ne les tient plus. Elle attrape l'un, et l'autre disparaît. Ils ne jouent plus au même endroit. On les reprend, les deux. Je ne veux pas choisir. Tu les poses comment, sur le siège ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le châle glisse sur le vinyle chaud. C'est trop lisse, ici. Le hérisson part vers l'allée, rond. Le renard se faufile sous le siège. Le châle ne les tient plus. Elle attrape l'un, et l'autre disparaît. Ils ne jouent plus au même endroit. Attrape-les ensemble, pas l'un après l'autre. Je ne veux pas choisir. Tu les poses comment, sur le siège ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -3988,7 +3988,7 @@
 enfant-f|Le châle ne les tient plus.
 narrateur|Elle attrape l'un, et l'autre disparaît.
 maman|Ils ne jouent plus au même endroit.
-papa|On les reprend, les deux.
+papa|Attrape-les ensemble, pas l'un après l'autre.
 enfant-f|Je ne veux pas choisir.
 papa|Tu les poses comment, sur le siège ?</t>
         </is>
@@ -4402,17 +4402,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Un brin de laine bleue reste au chaud. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, rond et fin.</t>
+          <t>La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Un pli bleu tient le creux, tiède. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, rond et fin.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Un brin de laine bleue reste au chaud. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, rond et fin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Un pli bleu tient le creux, tiède. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, rond et fin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Un brin de laine bleue reste au chaud. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, rond et fin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Un pli bleu tient le creux, tiède. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, rond et fin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4554,7 +4554,7 @@
 enfant-f|Plus personne ne roule.
 papa|Ils ont la même pente, jusqu'au bout.
 maman|Le chauffage ronronne, bas.
-narrateur|Un brin de laine bleue reste au chaud.
+narrateur|Un pli bleu tient le creux, tiède.
 narrateur|Le souffle de Chouchou dessine le noir.
 enfant-f|Puis le blanc.
 narrateur|Deux silhouettes restent dans la buée, rond et fin.</t>
@@ -4773,17 +4773,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Ça sent le beurre, un peu. Un brin de laine bleue reste au chaud. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, près du bleu.</t>
+          <t>La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Le beurre reste, même dans le noir. La laine sent la maison, près du beurre. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, près du bleu.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Ça sent le beurre, un peu. Un brin de laine bleue reste au chaud. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, près du bleu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Le beurre reste, même dans le noir. La laine sent la maison, près du beurre. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, près du bleu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Ça sent le beurre, un peu. Un brin de laine bleue reste au chaud. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, près du bleu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Le beurre reste, même dans le noir. La laine sent la maison, près du beurre. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, près du bleu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4924,8 +4924,8 @@
           <t>narrateur|La maison-boîte regarde la vitre, droit.
 enfant-f|Chacun sa fenêtre, même noir.
 papa|Deux chambres, un seul tunnel.
-maman|Ça sent le beurre, un peu.
-narrateur|Un brin de laine bleue reste au chaud.
+maman|Le beurre reste, même dans le noir.
+narrateur|La laine sent la maison, près du beurre.
 narrateur|Le verre devient noir, puis blanc.
 enfant-f|On est arrivés, presque.
 narrateur|Un flocon se pose au couvercle, près du bleu.</t>
@@ -5144,17 +5144,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Un brin de laine bleue reste au chaud. Le tunnel avale le wagon, une minute. Je vous ai gardés. La neige frappe le vinyle, et la lampe jaune revient.</t>
+          <t>La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Un coin bleu reste collé au dossier. Le tunnel avale le wagon, une minute. Je vous ai gardés. La neige frappe le vinyle, et la lampe jaune revient.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Un brin de laine bleue reste au chaud. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; frappe le vinyle, et la lampe jaune revient.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Un coin bleu reste collé au dossier. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; frappe le vinyle, et la lampe jaune revient.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Un brin de laine bleue reste au chaud. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis&gt;neige&lt;/emphasis&gt; frappe le vinyle, et la lampe jaune revient.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Un coin bleu reste collé au dossier. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis&gt;neige&lt;/emphasis&gt; frappe le vinyle, et la lampe jaune revient.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5296,7 +5296,7 @@
 enfant-f|Vous n'êtes plus sous le siège.
 papa|Ils ont voyagé à la même hauteur.
 maman|La banquette redevient un lit.
-narrateur|Un brin de laine bleue reste au chaud.
+narrateur|Un coin bleu reste collé au dossier.
 narrateur|Le tunnel avale le wagon, une minute.
 enfant-f|Je vous ai gardés.
 narrateur|La neige frappe le vinyle, et la lampe jaune revient.</t>
@@ -5900,17 +5900,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Un brin de laine bleue reste au chaud. Le noir presse un peu les oreilles. Puis la lumière revient. La neige entre par la fente, fine comme l'eau du pont.</t>
+          <t>Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Le bleu du châle chauffe le col. Le noir presse un peu les oreilles. Puis la lumière revient. La neige entre par la fente, fine comme l'eau du pont.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Un brin de laine bleue reste au chaud. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; entre par la fente, fine comme l'eau du pont.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Le bleu du châle chauffe le col. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; entre par la fente, fine comme l'eau du pont.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Un brin de laine bleue reste au chaud. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis&gt;neige&lt;/emphasis&gt; entre par la fente, fine comme l'eau du pont.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Le bleu du châle chauffe le col. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis&gt;neige&lt;/emphasis&gt; entre par la fente, fine comme l'eau du pont.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6052,7 +6052,7 @@
 enfant-f|Vous l'avez entendu, tous les deux.
 papa|Tes bras ont fait le wagon.
 maman|Le soufflet se tait, enfin.
-narrateur|Un brin de laine bleue reste au chaud.
+narrateur|Le bleu du châle chauffe le col.
 narrateur|Le noir presse un peu les oreilles.
 enfant-f|Puis la lumière revient.
 narrateur|La neige entre par la fente, fine comme l'eau du pont.</t>
@@ -6271,17 +6271,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Un brin de laine bleue reste au chaud. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de neige reste sur le fer, blanc comme le quai.</t>
+          <t>La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Un carré bleu reste sur les genoux. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de neige reste sur le fer, blanc comme le quai.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Un brin de laine bleue reste au chaud. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; reste sur le fer, blanc comme le quai.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Un carré bleu reste sur les genoux. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; reste sur le fer, blanc comme le quai.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Un brin de laine bleue reste au chaud. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis&gt;neige&lt;/emphasis&gt; reste sur le fer, blanc comme le quai.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Un carré bleu reste sur les genoux. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis&gt;neige&lt;/emphasis&gt; reste sur le fer, blanc comme le quai.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6423,7 +6423,7 @@
 enfant-f|Votre quai a vu le noir.
 papa|La marche était à toi, un moment.
 maman|Le joint ne les a pas pris.
-narrateur|Un brin de laine bleue reste au chaud.
+narrateur|Un carré bleu reste sur les genoux.
 narrateur|Le tunnel passe sous leurs pattes.
 enfant-f|On est des voyageurs, vraiment.
 narrateur|Un peu de neige reste sur le fer, blanc comme le quai.</t>
@@ -6642,17 +6642,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Un brin de laine bleue reste au chaud. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La neige allume le couloir, comme la lampe du quai.</t>
+          <t>Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Le châle retombe, tiède contre le verre. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La neige allume le couloir, comme la lampe du quai.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Un brin de laine bleue reste au chaud. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; allume le couloir, comme la lampe du quai.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Le châle retombe, tiède contre le verre. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; allume le couloir, comme la lampe du quai.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Un brin de laine bleue reste au chaud. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis&gt;neige&lt;/emphasis&gt; allume le couloir, comme la lampe du quai.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Le châle retombe, tiède contre le verre. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis&gt;neige&lt;/emphasis&gt; allume le couloir, comme la lampe du quai.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6794,7 +6794,7 @@
 enfant-f|On a attendu, puis on a vu.
 papa|Le calme t'a laissé la place.
 maman|La vitre du passage tient.
-narrateur|Un brin de laine bleue reste au chaud.
+narrateur|Le châle retombe, tiède contre le verre.
 narrateur|Le noir arrive sans danser, cette fois.
 enfant-f|Vous l'avez, tous les deux.
 narrateur|La neige allume le couloir, comme la lampe du quai.</t>
@@ -7578,17 +7578,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>La boîte penche dans le filet, clic. Votre cabine, trop penchée ! Le hérisson glisse au fond, lourd. Le renard racle le rebord, mince. Ils ne jouent plus au même endroit. Chouchou se dresse sur la pointe, déçue. Le fer ne les tient pas. On les reprend, les deux. Une miette tombe à travers une maille. Tu les gardes comment, dans le filet ?</t>
+          <t>La boîte penche dans le filet, clic. Votre cabine, trop penchée ! Le hérisson glisse au fond, lourd. Le renard racle le rebord, mince. Ils ne jouent plus au même endroit. Chouchou se dresse sur la pointe, déçue. Le fer ne les tient pas. On les reprend, sans en laisser un. Une miette tombe à travers une maille. Tu les gardes comment, dans le filet ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La boîte penche dans le &lt;emphasis level="moderate"&gt;filet&lt;/emphasis&gt;, clic. Votre cabine, trop penchée ! Le hérisson glisse au fond, lourd. Le renard racle le rebord, mince. Ils ne jouent plus au même endroit. Chouchou se dresse sur la pointe, déçue. Le fer ne les tient pas. On les reprend, les deux. Une miette tombe à travers une maille. Tu les gardes comment, dans le filet ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La boîte penche dans le &lt;emphasis level="moderate"&gt;filet&lt;/emphasis&gt;, clic. Votre cabine, trop penchée ! Le hérisson glisse au fond, lourd. Le renard racle le rebord, mince. Ils ne jouent plus au même endroit. Chouchou se dresse sur la pointe, déçue. Le fer ne les tient pas. On les reprend, sans en laisser un. Une miette tombe à travers une maille. Tu les gardes comment, dans le filet ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;La boîte penche dans le &lt;emphasis&gt;filet&lt;/emphasis&gt;, clic. Votre cabine, trop penchée ! Le hérisson glisse au fond, lourd. Le renard racle le rebord, mince. Ils ne jouent plus au même endroit. Chouchou se dresse sur la pointe, déçue. Le fer ne les tient pas. On les reprend, les deux. Une miette tombe à travers une maille. Tu les gardes comment, dans le filet ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;La boîte penche dans le &lt;emphasis&gt;filet&lt;/emphasis&gt;, clic. Votre cabine, trop penchée ! Le hérisson glisse au fond, lourd. Le renard racle le rebord, mince. Ils ne jouent plus au même endroit. Chouchou se dresse sur la pointe, déçue. Le fer ne les tient pas. On les reprend, sans en laisser un. Une miette tombe à travers une maille. Tu les gardes comment, dans le filet ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -7733,7 +7733,7 @@
 enfant-f|Ils ne jouent plus au même endroit.
 narrateur|Chouchou se dresse sur la pointe, déçue.
 maman|Le fer ne les tient pas.
-papa|On les reprend, les deux.
+papa|On les reprend, sans en laisser un.
 narrateur|Une miette tombe à travers une maille.
 papa|Tu les gardes comment, dans le filet ?</t>
         </is>
@@ -8518,17 +8518,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Une miette de biscuit dort au bord. Le noir entre, puis s'en va. De la neige, sur le métal. Un flocon reste au fer, près du clic.</t>
+          <t>Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Une miette sucrée reste au couvercle. Le noir entre, puis s'en va. De la neige, sur le métal. Un flocon reste au fer, près du clic.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Une miette de biscuit dort au bord. Le noir entre, puis s'en va. De la &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, près du clic.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Une miette sucrée reste au couvercle. Le noir entre, puis s'en va. De la &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, près du clic.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Une miette de biscuit dort au bord. Le noir entre, puis s'en va. De la &lt;emphasis&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, près du clic.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Une miette sucrée reste au couvercle. Le noir entre, puis s'en va. De la &lt;emphasis&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, près du clic.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8670,7 +8670,7 @@
 enfant-f|Vous voyez le trou, tous les deux ?
 papa|Deux places, une seule cabine.
 maman|Le filet les a gardés.
-narrateur|Une miette de biscuit dort au bord.
+narrateur|Une miette sucrée reste au couvercle.
 narrateur|Le noir entre, puis s'en va.
 enfant-f|De la neige, sur le métal.
 narrateur|Un flocon reste au fer, près du clic.</t>
@@ -8889,17 +8889,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Une miette de biscuit dort au bord. Le noir frappe le verre, un instant. On l'a vu, ensemble. La neige éclaire le manteau, et le couvercle.</t>
+          <t>Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Une odeur de beurre reste au métal. Le noir frappe le verre, un instant. On l'a vu, ensemble. La neige éclaire le manteau, et le couvercle.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Une miette de biscuit dort au bord. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le couvercle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Une odeur de beurre reste au métal. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le couvercle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Une miette de biscuit dort au bord. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le couvercle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Une odeur de beurre reste au métal. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le couvercle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9041,7 +9041,7 @@
 enfant-f|Vous êtes plus près, maintenant.
 papa|Tu les as repris tous les deux.
 maman|Le filet peut attendre, vide.
-narrateur|Une miette de biscuit dort au bord.
+narrateur|Une odeur de beurre reste au métal.
 narrateur|Le noir frappe le verre, un instant.
 enfant-f|On l'a vu, ensemble.
 narrateur|La neige éclaire le manteau, et le couvercle.</t>
@@ -9076,17 +9076,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>La boîte part vers l'allée, toc. Votre maison roule ! Le hérisson bute le couvercle, lourd. Le renard glisse sous le dossier, fin. Un dedans, un dessous, ce n'est pas juste. Chouchou a les mains trop petites, un instant. Le chauffage les emporte. On les reprend, les deux. Le vinyle sent le chaud, trop glissant. Tu les poses comment, sur le siège ?</t>
+          <t>La boîte part vers l'allée, toc. Votre maison roule ! Le hérisson bute le couvercle, lourd. Le renard glisse sous le dossier, fin. Un dedans, un dessous, ce n'est pas juste. Chouchou a les mains trop petites, un instant. Le chauffage les emporte. On les rattrape, tous les deux. Le vinyle sent le chaud, trop glissant. Tu les poses comment, sur le siège ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La boîte part vers l'allée, toc. Votre maison roule ! Le hérisson bute le couvercle, lourd. Le renard glisse sous le dossier, fin. Un dedans, un dessous, ce n'est pas juste. Chouchou a les mains trop petites, un instant. Le chauffage les emporte. On les reprend, les deux. Le vinyle sent le chaud, trop glissant. Tu les poses comment, sur le siège ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La boîte part vers l'allée, toc. Votre maison roule ! Le hérisson bute le couvercle, lourd. Le renard glisse sous le dossier, fin. Un dedans, un dessous, ce n'est pas juste. Chouchou a les mains trop petites, un instant. Le chauffage les emporte. On les rattrape, tous les deux. Le vinyle sent le chaud, trop glissant. Tu les poses comment, sur le siège ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;La boîte part vers l'allée, toc. Votre maison roule ! Le hérisson bute le couvercle, lourd. Le renard glisse sous le dossier, fin. Un dedans, un dessous, ce n'est pas juste. Chouchou a les mains trop petites, un instant. Le chauffage les emporte. On les reprend, les deux. Le vinyle sent le chaud, trop glissant. Tu les poses comment, sur le siège ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;La boîte part vers l'allée, toc. Votre maison roule ! Le hérisson bute le couvercle, lourd. Le renard glisse sous le dossier, fin. Un dedans, un dessous, ce n'est pas juste. Chouchou a les mains trop petites, un instant. Le chauffage les emporte. On les rattrape, tous les deux. Le vinyle sent le chaud, trop glissant. Tu les poses comment, sur le siège ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9231,7 +9231,7 @@
 enfant-f|Un dedans, un dessous, ce n'est pas juste.
 narrateur|Chouchou a les mains trop petites, un instant.
 maman|Le chauffage les emporte.
-papa|On les reprend, les deux.
+papa|On les rattrape, tous les deux.
 narrateur|Le vinyle sent le chaud, trop glissant.
 papa|Tu les poses comment, sur le siège ?</t>
         </is>
@@ -9645,17 +9645,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Une miette de biscuit dort au bord. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, dans la cabine.</t>
+          <t>La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Une miette brille dans la buée. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, dans la cabine.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Une miette de biscuit dort au bord. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, dans la cabine.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Une miette brille dans la buée. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, dans la cabine.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Une miette de biscuit dort au bord. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, dans la cabine.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Une miette brille dans la buée. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, dans la cabine.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9797,7 +9797,7 @@
 enfant-f|Plus personne ne roule.
 papa|Ils ont la même pente, jusqu'au bout.
 maman|Le chauffage ronronne, bas.
-narrateur|Une miette de biscuit dort au bord.
+narrateur|Une miette brille dans la buée.
 narrateur|Le souffle de Chouchou dessine le noir.
 enfant-f|Puis le blanc.
 narrateur|Deux silhouettes restent dans la buée, dans la cabine.</t>
@@ -9832,17 +9832,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Votre maison, face à la vitre. Elle ouvre la boîte, vers le verre froid. Le hérisson garde le coin gauche. Le renard garde le coin droit. Chacun sa fenêtre, dans la même maison. Deux chambres, une seule porte. Ça sent le beurre, un peu. Le couvercle fait deux petites places. Le tunnel va frapper le verre.</t>
+          <t>Votre maison, face à la vitre. Elle ouvre la boîte, vers le verre froid. Le hérisson garde le coin gauche. Le renard garde le coin droit. Chacun sa fenêtre, dans la même maison. Deux chambres, une seule porte. Ça sent le beurre, ici. Le couvercle fait deux petites places. Le tunnel va frapper le verre.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Votre &lt;emphasis level="moderate"&gt;maison&lt;/emphasis&gt;, face à la vitre. Elle ouvre la boîte, vers le verre froid. Le hérisson garde le coin gauche. Le renard garde le coin droit. Chacun sa fenêtre, dans la même maison. Deux chambres, une seule porte. Ça sent le beurre, un peu. Le couvercle fait deux petites places. Le tunnel va frapper le verre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Votre &lt;emphasis level="moderate"&gt;maison&lt;/emphasis&gt;, face à la vitre. Elle ouvre la boîte, vers le verre froid. Le hérisson garde le coin gauche. Le renard garde le coin droit. Chacun sa fenêtre, dans la même maison. Deux chambres, une seule porte. Ça sent le beurre, ici. Le couvercle fait deux petites places. Le tunnel va frapper le verre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Votre &lt;emphasis&gt;maison&lt;/emphasis&gt;, face à la vitre. Elle ouvre la boîte, vers le verre froid. Le hérisson garde le coin gauche. Le renard garde le coin droit. Chacun sa fenêtre, dans la même maison. Deux chambres, une seule porte. Ça sent le beurre, un peu. Le couvercle fait deux petites places. Le tunnel va frapper le verre. [pause]</t>
+          <t>Votre &lt;emphasis&gt;maison&lt;/emphasis&gt;, face à la vitre. Elle ouvre la boîte, vers le verre froid. Le hérisson garde le coin gauche. Le renard garde le coin droit. Chacun sa fenêtre, dans la même maison. Deux chambres, une seule porte. Ça sent le beurre, ici. Le couvercle fait deux petites places. Le tunnel va frapper le verre. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -9982,7 +9982,7 @@
 narrateur|Le renard garde le coin droit.
 enfant-f|Chacun sa fenêtre, dans la même maison.
 papa|Deux chambres, une seule porte.
-maman|Ça sent le beurre, un peu.
+maman|Ça sent le beurre, ici.
 narrateur|Le couvercle fait deux petites places.
 enfant-f|Le tunnel va frapper le verre.</t>
         </is>
@@ -10016,17 +10016,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Ça sent le beurre, un peu. Une miette de biscuit dort au bord. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, sucré.</t>
+          <t>La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Le couvercle sent le goûter. Le couvercle garde une odeur de beurre. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, sucré.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Ça sent le beurre, un peu. Une miette de biscuit dort au bord. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, sucré.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Le couvercle sent le goûter. Le couvercle garde une odeur de beurre. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, sucré.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Ça sent le beurre, un peu. Une miette de biscuit dort au bord. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, sucré.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Le couvercle sent le goûter. Le couvercle garde une odeur de beurre. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose au couvercle, sucré.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10167,8 +10167,8 @@
           <t>narrateur|La maison-boîte regarde la vitre, droit.
 enfant-f|Chacun sa fenêtre, même noir.
 papa|Deux chambres, un seul tunnel.
-maman|Ça sent le beurre, un peu.
-narrateur|Une miette de biscuit dort au bord.
+maman|Le couvercle sent le goûter.
+narrateur|Le couvercle garde une odeur de beurre.
 narrateur|Le verre devient noir, puis blanc.
 enfant-f|On est arrivés, presque.
 narrateur|Un flocon se pose au couvercle, sucré.</t>
@@ -10387,17 +10387,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Une miette de biscuit dort au bord. Le tunnel avale le wagon, une minute. Je vous ai gardés. La neige frappe le vinyle, près de la boîte.</t>
+          <t>La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Une miette roule, puis s'arrête. Le tunnel avale le wagon, une minute. Je vous ai gardés. La neige frappe le vinyle, près de la boîte.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Une miette de biscuit dort au bord. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; frappe le vinyle, près de la boîte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Une miette roule, puis s'arrête. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; frappe le vinyle, près de la boîte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Une miette de biscuit dort au bord. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis&gt;neige&lt;/emphasis&gt; frappe le vinyle, près de la boîte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Une miette roule, puis s'arrête. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis&gt;neige&lt;/emphasis&gt; frappe le vinyle, près de la boîte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10539,7 +10539,7 @@
 enfant-f|Vous n'êtes plus sous le siège.
 papa|Ils ont voyagé à la même hauteur.
 maman|La banquette redevient un lit.
-narrateur|Une miette de biscuit dort au bord.
+narrateur|Une miette roule, puis s'arrête.
 narrateur|Le tunnel avale le wagon, une minute.
 enfant-f|Je vous ai gardés.
 narrateur|La neige frappe le vinyle, près de la boîte.</t>
@@ -11143,17 +11143,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Une miette de biscuit dort au bord. Le noir presse un peu les oreilles. Puis la lumière revient. La neige entre par la fente, fine, sur le métal.</t>
+          <t>Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Le clic de la boîte se tait, sucré. Le noir presse un peu les oreilles. Puis la lumière revient. La neige entre par la fente, fine, sur le métal.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Une miette de biscuit dort au bord. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; entre par la fente, fine, sur le métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Le clic de la boîte se tait, sucré. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; entre par la fente, fine, sur le métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Une miette de biscuit dort au bord. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis&gt;neige&lt;/emphasis&gt; entre par la fente, fine, sur le métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Le clic de la boîte se tait, sucré. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis&gt;neige&lt;/emphasis&gt; entre par la fente, fine, sur le métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11295,7 +11295,7 @@
 enfant-f|Vous l'avez entendu, tous les deux.
 papa|Tes bras ont fait le wagon.
 maman|Le soufflet se tait, enfin.
-narrateur|Une miette de biscuit dort au bord.
+narrateur|Le clic de la boîte se tait, sucré.
 narrateur|Le noir presse un peu les oreilles.
 enfant-f|Puis la lumière revient.
 narrateur|La neige entre par la fente, fine, sur le métal.</t>
@@ -11514,17 +11514,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Une miette de biscuit dort au bord. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de neige reste sur le fer, et sur le couvercle.</t>
+          <t>La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Une miette reste sur le genou. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de neige reste sur le fer, et sur le couvercle.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Une miette de biscuit dort au bord. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; reste sur le fer, et sur le couvercle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Une miette reste sur le genou. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; reste sur le fer, et sur le couvercle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Une miette de biscuit dort au bord. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis&gt;neige&lt;/emphasis&gt; reste sur le fer, et sur le couvercle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Une miette reste sur le genou. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis&gt;neige&lt;/emphasis&gt; reste sur le fer, et sur le couvercle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11666,7 +11666,7 @@
 enfant-f|Votre quai a vu le noir.
 papa|La marche était à toi, un moment.
 maman|Le joint ne les a pas pris.
-narrateur|Une miette de biscuit dort au bord.
+narrateur|Une miette reste sur le genou.
 narrateur|Le tunnel passe sous leurs pattes.
 enfant-f|On est des voyageurs, vraiment.
 narrateur|Un peu de neige reste sur le fer, et sur le couvercle.</t>
@@ -11885,17 +11885,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Une miette de biscuit dort au bord. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La neige allume le couloir, et le clic se tait.</t>
+          <t>Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. L'odeur de beurre se tait, dans la cabine. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La neige allume le couloir, et le clic se tait.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Une miette de biscuit dort au bord. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; allume le couloir, et le clic se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. L'odeur de beurre se tait, dans la cabine. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; allume le couloir, et le clic se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Une miette de biscuit dort au bord. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis&gt;neige&lt;/emphasis&gt; allume le couloir, et le clic se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. L'odeur de beurre se tait, dans la cabine. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis&gt;neige&lt;/emphasis&gt; allume le couloir, et le clic se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12037,7 +12037,7 @@
 enfant-f|On a attendu, puis on a vu.
 papa|Le calme t'a laissé la place.
 maman|La vitre du passage tient.
-narrateur|Une miette de biscuit dort au bord.
+narrateur|L'odeur de beurre se tait, dans la cabine.
 narrateur|Le noir arrive sans danser, cette fois.
 enfant-f|Vous l'avez, tous les deux.
 narrateur|La neige allume le couloir, et le clic se tait.</t>
@@ -13761,17 +13761,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Le nœud de laine reste un peu tiède. Le noir entre, puis s'en va. De la neige, sur le métal. Un flocon reste au fer, accroché à la ficelle.</t>
+          <t>Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Le nœud frotte le fer, tiède. Le noir entre, puis s'en va. De la neige, sur le métal. Un flocon reste au fer, accroché à la ficelle.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Le nœud de laine reste un peu tiède. Le noir entre, puis s'en va. De la &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, accroché à la ficelle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Le nœud frotte le fer, tiède. Le noir entre, puis s'en va. De la &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, accroché à la ficelle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Le nœud de laine reste un peu tiède. Le noir entre, puis s'en va. De la &lt;emphasis&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, accroché à la ficelle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couvercle tremble, puis s'ouvre un peu. Vous voyez le trou, tous les deux ? Deux places, une seule cabine. Le filet les a gardés. Le nœud frotte le fer, tiède. Le noir entre, puis s'en va. De la &lt;emphasis&gt;neige&lt;/emphasis&gt;, sur le métal. Un flocon reste au fer, accroché à la ficelle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13913,7 +13913,7 @@
 enfant-f|Vous voyez le trou, tous les deux ?
 papa|Deux places, une seule cabine.
 maman|Le filet les a gardés.
-narrateur|Le nœud de laine reste un peu tiède.
+narrateur|Le nœud frotte le fer, tiède.
 narrateur|Le noir entre, puis s'en va.
 enfant-f|De la neige, sur le métal.
 narrateur|Un flocon reste au fer, accroché à la ficelle.</t>
@@ -14132,17 +14132,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Le nœud de laine reste un peu tiède. Le noir frappe le verre, un instant. On l'a vu, ensemble. La neige éclaire le manteau, et le poignet.</t>
+          <t>Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. La ficelle chauffe le poignet. Le noir frappe le verre, un instant. On l'a vu, ensemble. La neige éclaire le manteau, et le poignet.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Le nœud de laine reste un peu tiède. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le poignet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. La ficelle chauffe le poignet. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le poignet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. Le nœud de laine reste un peu tiède. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le poignet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ses bras baissent un peu, vers la vitre. Vous êtes plus près, maintenant. Tu les as repris tous les deux. Le filet peut attendre, vide. La ficelle chauffe le poignet. Le noir frappe le verre, un instant. On l'a vu, ensemble. La &lt;emphasis&gt;neige&lt;/emphasis&gt; éclaire le manteau, et le poignet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14284,7 +14284,7 @@
 enfant-f|Vous êtes plus près, maintenant.
 papa|Tu les as repris tous les deux.
 maman|Le filet peut attendre, vide.
-narrateur|Le nœud de laine reste un peu tiède.
+narrateur|La ficelle chauffe le poignet.
 narrateur|Le noir frappe le verre, un instant.
 enfant-f|On l'a vu, ensemble.
 narrateur|La neige éclaire le manteau, et le poignet.</t>
@@ -14319,17 +14319,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>La ficelle fuit sous le dossier, vive. Vous vous cachez ! Le hérisson reste coincé au bord, rond. Le renard tire le nœud vers l'ombre. Je ne chasse pas l'un sans l'autre. Elle s'agenouille, le cœur un peu lourd. Le siège les sépare. On les reprend, les deux. La laine racle le vinyle, puis se tait. Tu les poses comment, sur le siège ?</t>
+          <t>La ficelle fuit sous le dossier, vive. Vous vous cachez ! Le hérisson reste coincé au bord, rond. Le renard tire le nœud vers l'ombre. Je ne chasse pas l'un sans l'autre. Elle s'agenouille, le cœur un peu lourd. Le siège les sépare. Ramène le nœud, avec les deux. La laine racle le vinyle, puis se tait. Tu les poses comment, sur le siège ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La ficelle fuit sous le dossier, vive. Vous vous cachez ! Le hérisson reste coincé au bord, rond. Le renard tire le nœud vers l'ombre. Je ne chasse pas l'un sans l'autre. Elle s'agenouille, le cœur un peu lourd. Le siège les sépare. On les reprend, les deux. La laine racle le vinyle, puis se tait. Tu les poses comment, sur le siège ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La ficelle fuit sous le dossier, vive. Vous vous cachez ! Le hérisson reste coincé au bord, rond. Le renard tire le nœud vers l'ombre. Je ne chasse pas l'un sans l'autre. Elle s'agenouille, le cœur un peu lourd. Le siège les sépare. Ramène le nœud, avec les deux. La laine racle le vinyle, puis se tait. Tu les poses comment, sur le siège ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;La ficelle fuit sous le dossier, vive. Vous vous cachez ! Le hérisson reste coincé au bord, rond. Le renard tire le nœud vers l'ombre. Je ne chasse pas l'un sans l'autre. Elle s'agenouille, le cœur un peu lourd. Le siège les sépare. On les reprend, les deux. La laine racle le vinyle, puis se tait. Tu les poses comment, sur le siège ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;La ficelle fuit sous le dossier, vive. Vous vous cachez ! Le hérisson reste coincé au bord, rond. Le renard tire le nœud vers l'ombre. Je ne chasse pas l'un sans l'autre. Elle s'agenouille, le cœur un peu lourd. Le siège les sépare. Ramène le nœud, avec les deux. La laine racle le vinyle, puis se tait. Tu les poses comment, sur le siège ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14474,7 +14474,7 @@
 enfant-f|Je ne chasse pas l'un sans l'autre.
 narrateur|Elle s'agenouille, le cœur un peu lourd.
 maman|Le siège les sépare.
-papa|On les reprend, les deux.
+papa|Ramène le nœud, avec les deux.
 narrateur|La laine racle le vinyle, puis se tait.
 papa|Tu les poses comment, sur le siège ?</t>
         </is>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Le nœud de laine reste un peu tiède. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, liées.</t>
+          <t>La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Le nœud tient le creux, tiède. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, liées.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Le nœud de laine reste un peu tiède. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, liées.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Le nœud tient le creux, tiède. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, liées.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Le nœud de laine reste un peu tiède. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, liées.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La vallée de laine s'arrête, face au verre. Plus personne ne roule. Ils ont la même pente, jusqu'au bout. Le chauffage ronronne, bas. Le nœud tient le creux, tiède. Le souffle de Chouchou dessine le noir. Puis le blanc. Deux silhouettes restent dans la buée, liées.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15040,7 +15040,7 @@
 enfant-f|Plus personne ne roule.
 papa|Ils ont la même pente, jusqu'au bout.
 maman|Le chauffage ronronne, bas.
-narrateur|Le nœud de laine reste un peu tiède.
+narrateur|Le nœud tient le creux, tiède.
 narrateur|Le souffle de Chouchou dessine le noir.
 enfant-f|Puis le blanc.
 narrateur|Deux silhouettes restent dans la buée, liées.</t>
@@ -15259,17 +15259,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Ça sent le beurre, un peu. Le nœud de laine reste un peu tiède. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose à l'anse, sur le nœud.</t>
+          <t>La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Le nœud sent le goûter, lui aussi. Un brin de ficelle reste à l'anse. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose à l'anse, sur le nœud.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Ça sent le beurre, un peu. Le nœud de laine reste un peu tiède. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose à l'anse, sur le nœud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Le nœud sent le goûter, lui aussi. Un brin de ficelle reste à l'anse. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose à l'anse, sur le nœud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Ça sent le beurre, un peu. Le nœud de laine reste un peu tiède. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose à l'anse, sur le nœud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La maison-boîte regarde la vitre, droit. Chacun sa fenêtre, même noir. Deux chambres, un seul tunnel. Le nœud sent le goûter, lui aussi. Un brin de ficelle reste à l'anse. Le verre devient noir, puis blanc. On est arrivés, presque. Un flocon se pose à l'anse, sur le nœud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15410,8 +15410,8 @@
           <t>narrateur|La maison-boîte regarde la vitre, droit.
 enfant-f|Chacun sa fenêtre, même noir.
 papa|Deux chambres, un seul tunnel.
-maman|Ça sent le beurre, un peu.
-narrateur|Le nœud de laine reste un peu tiède.
+maman|Le nœud sent le goûter, lui aussi.
+narrateur|Un brin de ficelle reste à l'anse.
 narrateur|Le verre devient noir, puis blanc.
 enfant-f|On est arrivés, presque.
 narrateur|Un flocon se pose à l'anse, sur le nœud.</t>
@@ -15630,17 +15630,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Le nœud de laine reste un peu tiède. Le tunnel avale le wagon, une minute. Je vous ai gardés. La neige frappe le vinyle, et le double nœud.</t>
+          <t>La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Le double nœud reste au dossier, tiède. Le tunnel avale le wagon, une minute. Je vous ai gardés. La neige frappe le vinyle, et le double nœud.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Le nœud de laine reste un peu tiède. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; frappe le vinyle, et le double nœud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Le double nœud reste au dossier, tiède. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; frappe le vinyle, et le double nœud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Le nœud de laine reste un peu tiède. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis&gt;neige&lt;/emphasis&gt; frappe le vinyle, et le double nœud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La ceinture de laine tient le dossier. Vous n'êtes plus sous le siège. Ils ont voyagé à la même hauteur. La banquette redevient un lit. Le double nœud reste au dossier, tiède. Le tunnel avale le wagon, une minute. Je vous ai gardés. La &lt;emphasis&gt;neige&lt;/emphasis&gt; frappe le vinyle, et le double nœud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -15782,7 +15782,7 @@
 enfant-f|Vous n'êtes plus sous le siège.
 papa|Ils ont voyagé à la même hauteur.
 maman|La banquette redevient un lit.
-narrateur|Le nœud de laine reste un peu tiède.
+narrateur|Le double nœud reste au dossier, tiède.
 narrateur|Le tunnel avale le wagon, une minute.
 enfant-f|Je vous ai gardés.
 narrateur|La neige frappe le vinyle, et le double nœud.</t>
@@ -16386,17 +16386,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Le nœud de laine reste un peu tiède. Le noir presse un peu les oreilles. Puis la lumière revient. La neige entre par la fente, fine, sur le pouce.</t>
+          <t>Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. La ficelle chauffe le pouce. Le noir presse un peu les oreilles. Puis la lumière revient. La neige entre par la fente, fine, sur le pouce.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Le nœud de laine reste un peu tiède. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; entre par la fente, fine, sur le pouce.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. La ficelle chauffe le pouce. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; entre par la fente, fine, sur le pouce.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. Le nœud de laine reste un peu tiède. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis&gt;neige&lt;/emphasis&gt; entre par la fente, fine, sur le pouce.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Son cœur et le train parlent ensemble. Vous l'avez entendu, tous les deux. Tes bras ont fait le wagon. Le soufflet se tait, enfin. La ficelle chauffe le pouce. Le noir presse un peu les oreilles. Puis la lumière revient. La &lt;emphasis&gt;neige&lt;/emphasis&gt; entre par la fente, fine, sur le pouce.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16538,7 +16538,7 @@
 enfant-f|Vous l'avez entendu, tous les deux.
 papa|Tes bras ont fait le wagon.
 maman|Le soufflet se tait, enfin.
-narrateur|Le nœud de laine reste un peu tiède.
+narrateur|La ficelle chauffe le pouce.
 narrateur|Le noir presse un peu les oreilles.
 enfant-f|Puis la lumière revient.
 narrateur|La neige entre par la fente, fine, sur le pouce.</t>
@@ -16757,17 +16757,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Le nœud de laine reste un peu tiède. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de neige reste sur le fer, près de la cheville.</t>
+          <t>La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Le nœud reste près de la cheville, tiède. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de neige reste sur le fer, près de la cheville.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Le nœud de laine reste un peu tiède. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; reste sur le fer, près de la cheville.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Le nœud reste près de la cheville, tiède. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; reste sur le fer, près de la cheville.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Le nœud de laine reste un peu tiède. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis&gt;neige&lt;/emphasis&gt; reste sur le fer, près de la cheville.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La marche vibre, puis s'endort. Votre quai a vu le noir. La marche était à toi, un moment. Le joint ne les a pas pris. Le nœud reste près de la cheville, tiède. Le tunnel passe sous leurs pattes. On est des voyageurs, vraiment. Un peu de &lt;emphasis&gt;neige&lt;/emphasis&gt; reste sur le fer, près de la cheville.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -16909,7 +16909,7 @@
 enfant-f|Votre quai a vu le noir.
 papa|La marche était à toi, un moment.
 maman|Le joint ne les a pas pris.
-narrateur|Le nœud de laine reste un peu tiède.
+narrateur|Le nœud reste près de la cheville, tiède.
 narrateur|Le tunnel passe sous leurs pattes.
 enfant-f|On est des voyageurs, vraiment.
 narrateur|Un peu de neige reste sur le fer, près de la cheville.</t>
@@ -17128,17 +17128,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Le nœud de laine reste un peu tiède. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La neige allume le couloir, et le poignet se tait.</t>
+          <t>Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Le nœud se tait contre le verre, tiède. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La neige allume le couloir, et le poignet se tait.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Le nœud de laine reste un peu tiède. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; allume le couloir, et le poignet se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Le nœud se tait contre le verre, tiède. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis level="moderate"&gt;neige&lt;/emphasis&gt; allume le couloir, et le poignet se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Le nœud de laine reste un peu tiède. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis&gt;neige&lt;/emphasis&gt; allume le couloir, et le poignet se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le plancher s'est tu, juste à temps. On a attendu, puis on a vu. Le calme t'a laissé la place. La vitre du passage tient. Le nœud se tait contre le verre, tiède. Le noir arrive sans danser, cette fois. Vous l'avez, tous les deux. La &lt;emphasis&gt;neige&lt;/emphasis&gt; allume le couloir, et le poignet se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17280,7 +17280,7 @@
 enfant-f|On a attendu, puis on a vu.
 papa|Le calme t'a laissé la place.
 maman|La vitre du passage tient.
-narrateur|Le nœud de laine reste un peu tiède.
+narrateur|Le nœud se tait contre le verre, tiède.
 narrateur|Le noir arrive sans danser, cette fois.
 enfant-f|Vous l'avez, tous les deux.
 narrateur|La neige allume le couloir, et le poignet se tait.</t>
@@ -17309,7 +17309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17359,6 +17359,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>